<commit_message>
Add May monthly projection sheet (calendar-day and business-day basis)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015f56A799NhnuL2TDwF4NVd
</commit_message>
<xml_diff>
--- a/조제내역_약가합계순.xlsx
+++ b/조제내역_약가합계순.xlsx
@@ -7,12 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-05-01~05-22" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-07-20~08-20" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5월 한달 환산" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-05-01~05-22" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-07-20~08-20" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-05-01~05-22'!$A$1:$P$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-07-20~08-20'!$A$1:$P$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'5월 한달 환산'!$A$8:$N$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-05-01~05-22'!$A$1:$P$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2026-07-20~08-20'!$A$1:$P$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.##"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +37,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,12 +72,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,6 +448,2676 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>조회 일수(05-01~05-22)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>5월 전체 일수</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>조회 영업일 수</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>5월 전체 영업일 수</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>일회성 기준(조제건수 이하는 환산 제외)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>영업일은 일요일, 5/1, 5/5, 5/25(대체공휴일) 휴무로 가정한 값입니다. 실제 휴무일에 맞게 노란 칸(B3, B4)을 고치면 전체가 다시 계산됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>약품명</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>약품코드</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>제약회사</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>약품단가</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>조제수량(1~22일)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>조제건수(1~22일)</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>약가합계(1~22일)</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>한달 조제수량(일수 기준)</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>한달 약가합계(일수 기준)</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>한달 조제수량(영업일 기준)</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>한달 약가합계(영업일 기준)</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>한달 조제건수(영업일 기준)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>프리그렐정</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>643304110</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>종근당</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>911</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>18684</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>17021124</v>
+      </c>
+      <c r="I9">
+        <f>IF(G9&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J9" s="5">
+        <f>IF(I9="",F9*$B$2/$B$1,F9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="5">
+        <f>IF(I9="",H9*$B$2/$B$1,H9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="5">
+        <f>IF(I9="",F9*$B$4/$B$3,F9)</f>
+        <v/>
+      </c>
+      <c r="M9" s="5">
+        <f>IF(I9="",H9*$B$4/$B$3,H9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="5">
+        <f>IF(I9="",G9*$B$4/$B$3,G9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>글리아티민연질캡슐</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>694000600</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>대웅바이오</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>33336</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>263</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>15867936</v>
+      </c>
+      <c r="I10">
+        <f>IF(G10&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J10" s="5">
+        <f>IF(I10="",F10*$B$2/$B$1,F10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="5">
+        <f>IF(I10="",H10*$B$2/$B$1,H10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="5">
+        <f>IF(I10="",F10*$B$4/$B$3,F10)</f>
+        <v/>
+      </c>
+      <c r="M10" s="5">
+        <f>IF(I10="",H10*$B$4/$B$3,H10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="5">
+        <f>IF(I10="",G10*$B$4/$B$3,G10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>비리어드정</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>625900040</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>길리어드</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>2501</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>3381</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>8455881</v>
+      </c>
+      <c r="I11">
+        <f>IF(G11&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J11" s="5">
+        <f>IF(I11="",F11*$B$2/$B$1,F11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="5">
+        <f>IF(I11="",H11*$B$2/$B$1,H11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="5">
+        <f>IF(I11="",F11*$B$4/$B$3,F11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="5">
+        <f>IF(I11="",H11*$B$4/$B$3,H11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="5">
+        <f>IF(I11="",G11*$B$4/$B$3,G11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>케이캡정50밀리그램</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>640007270</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>에이치케이이노엔</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>1299</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>6310</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>187</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>8196690</v>
+      </c>
+      <c r="I12">
+        <f>IF(G12&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J12" s="5">
+        <f>IF(I12="",F12*$B$2/$B$1,F12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="5">
+        <f>IF(I12="",H12*$B$2/$B$1,H12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="5">
+        <f>IF(I12="",F12*$B$4/$B$3,F12)</f>
+        <v/>
+      </c>
+      <c r="M12" s="5">
+        <f>IF(I12="",H12*$B$4/$B$3,H12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="5">
+        <f>IF(I12="",G12*$B$4/$B$3,G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>플라리스정</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>647802630</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>삼진제약</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>1077</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>7529</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>8108733</v>
+      </c>
+      <c r="I13">
+        <f>IF(G13&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J13" s="5">
+        <f>IF(I13="",F13*$B$2/$B$1,F13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>IF(I13="",H13*$B$2/$B$1,H13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="5">
+        <f>IF(I13="",F13*$B$4/$B$3,F13)</f>
+        <v/>
+      </c>
+      <c r="M13" s="5">
+        <f>IF(I13="",H13*$B$4/$B$3,H13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5">
+        <f>IF(I13="",G13*$B$4/$B$3,G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>카소비드정</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>648503130</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>신풍제약</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>3592</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>2136</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>7672512</v>
+      </c>
+      <c r="I14">
+        <f>IF(G14&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J14" s="5">
+        <f>IF(I14="",F14*$B$2/$B$1,F14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="5">
+        <f>IF(I14="",H14*$B$2/$B$1,H14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="5">
+        <f>IF(I14="",F14*$B$4/$B$3,F14)</f>
+        <v/>
+      </c>
+      <c r="M14" s="5">
+        <f>IF(I14="",H14*$B$4/$B$3,H14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="5">
+        <f>IF(I14="",G14*$B$4/$B$3,G14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>브레트라정</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>648501310</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>신풍제약</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>2904</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>2326</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>6754704</v>
+      </c>
+      <c r="I15">
+        <f>IF(G15&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J15" s="5">
+        <f>IF(I15="",F15*$B$2/$B$1,F15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="5">
+        <f>IF(I15="",H15*$B$2/$B$1,H15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="5">
+        <f>IF(I15="",F15*$B$4/$B$3,F15)</f>
+        <v/>
+      </c>
+      <c r="M15" s="5">
+        <f>IF(I15="",H15*$B$4/$B$3,H15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="5">
+        <f>IF(I15="",G15*$B$4/$B$3,G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>이지산트정10/10밀리그램</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>641906350</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>(주)보령</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>1063</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>6054</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>6435402</v>
+      </c>
+      <c r="I16">
+        <f>IF(G16&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J16" s="5">
+        <f>IF(I16="",F16*$B$2/$B$1,F16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="5">
+        <f>IF(I16="",H16*$B$2/$B$1,H16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="5">
+        <f>IF(I16="",F16*$B$4/$B$3,F16)</f>
+        <v/>
+      </c>
+      <c r="M16" s="5">
+        <f>IF(I16="",H16*$B$4/$B$3,H16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="5">
+        <f>IF(I16="",G16*$B$4/$B$3,G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>베믈리디정</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>625900120</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>길리어드</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>3139</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1872</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>5876208</v>
+      </c>
+      <c r="I17">
+        <f>IF(G17&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J17" s="5">
+        <f>IF(I17="",F17*$B$2/$B$1,F17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="5">
+        <f>IF(I17="",H17*$B$2/$B$1,H17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="5">
+        <f>IF(I17="",F17*$B$4/$B$3,F17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="5">
+        <f>IF(I17="",H17*$B$4/$B$3,H17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="5">
+        <f>IF(I17="",G17*$B$4/$B$3,G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>펜졸캡슐</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>643305980</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>(주)종근당</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>2264</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>2562</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>5800368</v>
+      </c>
+      <c r="I18">
+        <f>IF(G18&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J18" s="5">
+        <f>IF(I18="",F18*$B$2/$B$1,F18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="5">
+        <f>IF(I18="",H18*$B$2/$B$1,H18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="5">
+        <f>IF(I18="",F18*$B$4/$B$3,F18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="5">
+        <f>IF(I18="",H18*$B$4/$B$3,H18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="5">
+        <f>IF(I18="",G18*$B$4/$B$3,G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>유로박솜캡셀</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>654001440</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>아주약품</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>706</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>7932</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>5599992</v>
+      </c>
+      <c r="I19">
+        <f>IF(G19&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J19" s="5">
+        <f>IF(I19="",F19*$B$2/$B$1,F19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="5">
+        <f>IF(I19="",H19*$B$2/$B$1,H19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="5">
+        <f>IF(I19="",F19*$B$4/$B$3,F19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="5">
+        <f>IF(I19="",H19*$B$4/$B$3,H19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="5">
+        <f>IF(I19="",G19*$B$4/$B$3,G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>이지산트정10/5밀리그램</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>641906360</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>(주)보령</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>761</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>7133</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>5428213</v>
+      </c>
+      <c r="I20">
+        <f>IF(G20&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J20" s="5">
+        <f>IF(I20="",F20*$B$2/$B$1,F20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="5">
+        <f>IF(I20="",H20*$B$2/$B$1,H20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="5">
+        <f>IF(I20="",F20*$B$4/$B$3,F20)</f>
+        <v/>
+      </c>
+      <c r="M20" s="5">
+        <f>IF(I20="",H20*$B$4/$B$3,H20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="5">
+        <f>IF(I20="",G20*$B$4/$B$3,G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>엔트레스토필름코팅정50밀리그램</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>653602720</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>한국노바티스</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>1554</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>3340.5</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>5191137</v>
+      </c>
+      <c r="I21">
+        <f>IF(G21&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J21" s="5">
+        <f>IF(I21="",F21*$B$2/$B$1,F21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="5">
+        <f>IF(I21="",H21*$B$2/$B$1,H21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="5">
+        <f>IF(I21="",F21*$B$4/$B$3,F21)</f>
+        <v/>
+      </c>
+      <c r="M21" s="5">
+        <f>IF(I21="",H21*$B$4/$B$3,H21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="5">
+        <f>IF(I21="",G21*$B$4/$B$3,G21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>리피로우정20밀리그램</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>643300660</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>(주)종근당</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>707</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>6896</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>4875472</v>
+      </c>
+      <c r="I22">
+        <f>IF(G22&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J22" s="5">
+        <f>IF(I22="",F22*$B$2/$B$1,F22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="5">
+        <f>IF(I22="",H22*$B$2/$B$1,H22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="5">
+        <f>IF(I22="",F22*$B$4/$B$3,F22)</f>
+        <v/>
+      </c>
+      <c r="M22" s="5">
+        <f>IF(I22="",H22*$B$4/$B$3,H22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="5">
+        <f>IF(I22="",G22*$B$4/$B$3,G22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>엑시드캡슐150밀리그램</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>641601910</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>대웅제약</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>308</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>15740</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>159</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>4847920</v>
+      </c>
+      <c r="I23">
+        <f>IF(G23&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J23" s="5">
+        <f>IF(I23="",F23*$B$2/$B$1,F23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="5">
+        <f>IF(I23="",H23*$B$2/$B$1,H23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="5">
+        <f>IF(I23="",F23*$B$4/$B$3,F23)</f>
+        <v/>
+      </c>
+      <c r="M23" s="5">
+        <f>IF(I23="",H23*$B$4/$B$3,H23)</f>
+        <v/>
+      </c>
+      <c r="N23" s="5">
+        <f>IF(I23="",G23*$B$4/$B$3,G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>휴미라펜주40mg/0.4mL</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>624900271</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>한국애브비</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>284677</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>4839509</v>
+      </c>
+      <c r="I24">
+        <f>IF(G24&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J24" s="5">
+        <f>IF(I24="",F24*$B$2/$B$1,F24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="5">
+        <f>IF(I24="",H24*$B$2/$B$1,H24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="5">
+        <f>IF(I24="",F24*$B$4/$B$3,F24)</f>
+        <v/>
+      </c>
+      <c r="M24" s="5">
+        <f>IF(I24="",H24*$B$4/$B$3,H24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="5">
+        <f>IF(I24="",G24*$B$4/$B$3,G24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>구루치온정100mg</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2118202</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>영풍제약</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>6797</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>4757900</v>
+      </c>
+      <c r="I25">
+        <f>IF(G25&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J25" s="5">
+        <f>IF(I25="",F25*$B$2/$B$1,F25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="5">
+        <f>IF(I25="",H25*$B$2/$B$1,H25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="5">
+        <f>IF(I25="",F25*$B$4/$B$3,F25)</f>
+        <v/>
+      </c>
+      <c r="M25" s="5">
+        <f>IF(I25="",H25*$B$4/$B$3,H25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="5">
+        <f>IF(I25="",G25*$B$4/$B$3,G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>리피토정10밀리그램</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>073400340</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>비아트리스</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>638</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>7292</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>79</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>4652296</v>
+      </c>
+      <c r="I26">
+        <f>IF(G26&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J26" s="5">
+        <f>IF(I26="",F26*$B$2/$B$1,F26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="5">
+        <f>IF(I26="",H26*$B$2/$B$1,H26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="5">
+        <f>IF(I26="",F26*$B$4/$B$3,F26)</f>
+        <v/>
+      </c>
+      <c r="M26" s="5">
+        <f>IF(I26="",H26*$B$4/$B$3,H26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="5">
+        <f>IF(I26="",G26*$B$4/$B$3,G26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>19</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>베아셉트정5밀리그램</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>694001110</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>대웅바이오</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>1855</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>2466</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>4574430</v>
+      </c>
+      <c r="I27">
+        <f>IF(G27&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J27" s="5">
+        <f>IF(I27="",F27*$B$2/$B$1,F27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="5">
+        <f>IF(I27="",H27*$B$2/$B$1,H27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="5">
+        <f>IF(I27="",F27*$B$4/$B$3,F27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="5">
+        <f>IF(I27="",H27*$B$4/$B$3,H27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="5">
+        <f>IF(I27="",G27*$B$4/$B$3,G27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>탐스피드캡슐</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>647802310</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>삼진제약</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>465</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>9788</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>131</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>4551420</v>
+      </c>
+      <c r="I28">
+        <f>IF(G28&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J28" s="5">
+        <f>IF(I28="",F28*$B$2/$B$1,F28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="5">
+        <f>IF(I28="",H28*$B$2/$B$1,H28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="5">
+        <f>IF(I28="",F28*$B$4/$B$3,F28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="5">
+        <f>IF(I28="",H28*$B$4/$B$3,H28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="5">
+        <f>IF(I28="",G28*$B$4/$B$3,G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>21</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>플라빅스정75밀리그램</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>652101570</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>(주)한독</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>1081</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>4102</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>4434262</v>
+      </c>
+      <c r="I29">
+        <f>IF(G29&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J29" s="5">
+        <f>IF(I29="",F29*$B$2/$B$1,F29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="5">
+        <f>IF(I29="",H29*$B$2/$B$1,H29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="5">
+        <f>IF(I29="",F29*$B$4/$B$3,F29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="5">
+        <f>IF(I29="",H29*$B$4/$B$3,H29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="5">
+        <f>IF(I29="",G29*$B$4/$B$3,G29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>바이오탑하이포르테캡슐</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2120438</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>6274</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>4391800</v>
+      </c>
+      <c r="I30">
+        <f>IF(G30&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J30" s="5">
+        <f>IF(I30="",F30*$B$2/$B$1,F30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="5">
+        <f>IF(I30="",H30*$B$2/$B$1,H30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="5">
+        <f>IF(I30="",F30*$B$4/$B$3,F30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="5">
+        <f>IF(I30="",H30*$B$4/$B$3,H30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="5">
+        <f>IF(I30="",G30*$B$4/$B$3,G30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>23</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>로수젯정10/20밀리그램</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>643507270</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>한미약품</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>1093</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>3993</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>4367749</v>
+      </c>
+      <c r="I31">
+        <f>IF(G31&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J31" s="5">
+        <f>IF(I31="",F31*$B$2/$B$1,F31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="5">
+        <f>IF(I31="",H31*$B$2/$B$1,H31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="5">
+        <f>IF(I31="",F31*$B$4/$B$3,F31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="5">
+        <f>IF(I31="",H31*$B$4/$B$3,H31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="5">
+        <f>IF(I31="",G31*$B$4/$B$3,G31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>로수로드정10밀리그램</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>643305080</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>종근당</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>611</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>7128</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>4355208</v>
+      </c>
+      <c r="I32">
+        <f>IF(G32&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J32" s="5">
+        <f>IF(I32="",F32*$B$2/$B$1,F32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="5">
+        <f>IF(I32="",H32*$B$2/$B$1,H32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="5">
+        <f>IF(I32="",F32*$B$4/$B$3,F32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="5">
+        <f>IF(I32="",H32*$B$4/$B$3,H32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="5">
+        <f>IF(I32="",G32*$B$4/$B$3,G32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>25</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>펜넬캡슐</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>652300700</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>파마킹</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>312</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>13648</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>4258176</v>
+      </c>
+      <c r="I33">
+        <f>IF(G33&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J33" s="5">
+        <f>IF(I33="",F33*$B$2/$B$1,F33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="5">
+        <f>IF(I33="",H33*$B$2/$B$1,H33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="5">
+        <f>IF(I33="",F33*$B$4/$B$3,F33)</f>
+        <v/>
+      </c>
+      <c r="M33" s="5">
+        <f>IF(I33="",H33*$B$4/$B$3,H33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="5">
+        <f>IF(I33="",G33*$B$4/$B$3,G33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>26</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>유리토스정</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>668901520</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>(주)엘지화학</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>391</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>10576</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>4135216</v>
+      </c>
+      <c r="I34">
+        <f>IF(G34&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J34" s="5">
+        <f>IF(I34="",F34*$B$2/$B$1,F34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="5">
+        <f>IF(I34="",H34*$B$2/$B$1,H34)</f>
+        <v/>
+      </c>
+      <c r="L34" s="5">
+        <f>IF(I34="",F34*$B$4/$B$3,F34)</f>
+        <v/>
+      </c>
+      <c r="M34" s="5">
+        <f>IF(I34="",H34*$B$4/$B$3,H34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="5">
+        <f>IF(I34="",G34*$B$4/$B$3,G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>27</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>자큐보정20밀리그램</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>078600010</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>온코닉테라퓨틱스</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>911</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>4533</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>4129563</v>
+      </c>
+      <c r="I35">
+        <f>IF(G35&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J35" s="5">
+        <f>IF(I35="",F35*$B$2/$B$1,F35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="5">
+        <f>IF(I35="",H35*$B$2/$B$1,H35)</f>
+        <v/>
+      </c>
+      <c r="L35" s="5">
+        <f>IF(I35="",F35*$B$4/$B$3,F35)</f>
+        <v/>
+      </c>
+      <c r="M35" s="5">
+        <f>IF(I35="",H35*$B$4/$B$3,H35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="5">
+        <f>IF(I35="",G35*$B$4/$B$3,G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>28</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>글리아타민정</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>694000670</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>대웅바이오</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>8537</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>4063612</v>
+      </c>
+      <c r="I36">
+        <f>IF(G36&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J36" s="5">
+        <f>IF(I36="",F36*$B$2/$B$1,F36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="5">
+        <f>IF(I36="",H36*$B$2/$B$1,H36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="5">
+        <f>IF(I36="",F36*$B$4/$B$3,F36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="5">
+        <f>IF(I36="",H36*$B$4/$B$3,H36)</f>
+        <v/>
+      </c>
+      <c r="N36" s="5">
+        <f>IF(I36="",G36*$B$4/$B$3,G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>29</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>보령피나스테리드정5밀리그램</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>641902100</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>(주)보령</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>622</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>6384</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>3970848</v>
+      </c>
+      <c r="I37">
+        <f>IF(G37&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J37" s="5">
+        <f>IF(I37="",F37*$B$2/$B$1,F37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="5">
+        <f>IF(I37="",H37*$B$2/$B$1,H37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="5">
+        <f>IF(I37="",F37*$B$4/$B$3,F37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="5">
+        <f>IF(I37="",H37*$B$4/$B$3,H37)</f>
+        <v/>
+      </c>
+      <c r="N37" s="5">
+        <f>IF(I37="",G37*$B$4/$B$3,G37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>30</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>타그리소정80밀리그램</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>650700980</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>한국아스트라제네카</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>190108</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>5323024</v>
+      </c>
+      <c r="I38">
+        <f>IF(G38&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J38" s="5">
+        <f>IF(I38="",F38*$B$2/$B$1,F38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="5">
+        <f>IF(I38="",H38*$B$2/$B$1,H38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="5">
+        <f>IF(I38="",F38*$B$4/$B$3,F38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="5">
+        <f>IF(I38="",H38*$B$4/$B$3,H38)</f>
+        <v/>
+      </c>
+      <c r="N38" s="5">
+        <f>IF(I38="",G38*$B$4/$B$3,G38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>31</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>투톤네블정</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>671806950</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>대원제약</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>162</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>23554</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>3815748</v>
+      </c>
+      <c r="I39">
+        <f>IF(G39&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J39" s="5">
+        <f>IF(I39="",F39*$B$2/$B$1,F39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="5">
+        <f>IF(I39="",H39*$B$2/$B$1,H39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="5">
+        <f>IF(I39="",F39*$B$4/$B$3,F39)</f>
+        <v/>
+      </c>
+      <c r="M39" s="5">
+        <f>IF(I39="",H39*$B$4/$B$3,H39)</f>
+        <v/>
+      </c>
+      <c r="N39" s="5">
+        <f>IF(I39="",G39*$B$4/$B$3,G39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>32</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>로수젯정10/10밀리그램</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>643507260</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>한미약품</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>1087</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>3457</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>3757759</v>
+      </c>
+      <c r="I40">
+        <f>IF(G40&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J40" s="5">
+        <f>IF(I40="",F40*$B$2/$B$1,F40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="5">
+        <f>IF(I40="",H40*$B$2/$B$1,H40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="5">
+        <f>IF(I40="",F40*$B$4/$B$3,F40)</f>
+        <v/>
+      </c>
+      <c r="M40" s="5">
+        <f>IF(I40="",H40*$B$4/$B$3,H40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="5">
+        <f>IF(I40="",G40*$B$4/$B$3,G40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>33</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>케프라정500밀리그램</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>654100150</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>한국유씨비</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>693</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>5420.5</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>3756407</v>
+      </c>
+      <c r="I41">
+        <f>IF(G41&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J41" s="5">
+        <f>IF(I41="",F41*$B$2/$B$1,F41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="5">
+        <f>IF(I41="",H41*$B$2/$B$1,H41)</f>
+        <v/>
+      </c>
+      <c r="L41" s="5">
+        <f>IF(I41="",F41*$B$4/$B$3,F41)</f>
+        <v/>
+      </c>
+      <c r="M41" s="5">
+        <f>IF(I41="",H41*$B$4/$B$3,H41)</f>
+        <v/>
+      </c>
+      <c r="N41" s="5">
+        <f>IF(I41="",G41*$B$4/$B$3,G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>34</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>리바로젯정2/10밀리그램</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>644914960</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>제이더블유중외</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>1307</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>2809</v>
+      </c>
+      <c r="G42" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>3671363</v>
+      </c>
+      <c r="I42">
+        <f>IF(G42&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J42" s="5">
+        <f>IF(I42="",F42*$B$2/$B$1,F42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="5">
+        <f>IF(I42="",H42*$B$2/$B$1,H42)</f>
+        <v/>
+      </c>
+      <c r="L42" s="5">
+        <f>IF(I42="",F42*$B$4/$B$3,F42)</f>
+        <v/>
+      </c>
+      <c r="M42" s="5">
+        <f>IF(I42="",H42*$B$4/$B$3,H42)</f>
+        <v/>
+      </c>
+      <c r="N42" s="5">
+        <f>IF(I42="",G42*$B$4/$B$3,G42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>35</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>릭시아나정30밀리그램</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>680900180</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>한국다이이찌산쿄</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>2032</v>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>1745</v>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>3545840</v>
+      </c>
+      <c r="I43">
+        <f>IF(G43&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J43" s="5">
+        <f>IF(I43="",F43*$B$2/$B$1,F43)</f>
+        <v/>
+      </c>
+      <c r="K43" s="5">
+        <f>IF(I43="",H43*$B$2/$B$1,H43)</f>
+        <v/>
+      </c>
+      <c r="L43" s="5">
+        <f>IF(I43="",F43*$B$4/$B$3,F43)</f>
+        <v/>
+      </c>
+      <c r="M43" s="5">
+        <f>IF(I43="",H43*$B$4/$B$3,H43)</f>
+        <v/>
+      </c>
+      <c r="N43" s="5">
+        <f>IF(I43="",G43*$B$4/$B$3,G43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>36</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>펙수클루정40밀리그램</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>641607630</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>(주)대웅제약</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>901</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>3931</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>3541831</v>
+      </c>
+      <c r="I44">
+        <f>IF(G44&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J44" s="5">
+        <f>IF(I44="",F44*$B$2/$B$1,F44)</f>
+        <v/>
+      </c>
+      <c r="K44" s="5">
+        <f>IF(I44="",H44*$B$2/$B$1,H44)</f>
+        <v/>
+      </c>
+      <c r="L44" s="5">
+        <f>IF(I44="",F44*$B$4/$B$3,F44)</f>
+        <v/>
+      </c>
+      <c r="M44" s="5">
+        <f>IF(I44="",H44*$B$4/$B$3,H44)</f>
+        <v/>
+      </c>
+      <c r="N44" s="5">
+        <f>IF(I44="",G44*$B$4/$B$3,G44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>37</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>이지산트정10/20밀리그램</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>641906340</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>(주)보령</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>1074</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>3189</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>3424986</v>
+      </c>
+      <c r="I45">
+        <f>IF(G45&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J45" s="5">
+        <f>IF(I45="",F45*$B$2/$B$1,F45)</f>
+        <v/>
+      </c>
+      <c r="K45" s="5">
+        <f>IF(I45="",H45*$B$2/$B$1,H45)</f>
+        <v/>
+      </c>
+      <c r="L45" s="5">
+        <f>IF(I45="",F45*$B$4/$B$3,F45)</f>
+        <v/>
+      </c>
+      <c r="M45" s="5">
+        <f>IF(I45="",H45*$B$4/$B$3,H45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="5">
+        <f>IF(I45="",G45*$B$4/$B$3,G45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>38</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>딜라트렌에스알캡슐16밀리그램</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>643306410</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>(주)종근당</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>543</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>6108</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>3316684</v>
+      </c>
+      <c r="I46">
+        <f>IF(G46&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J46" s="5">
+        <f>IF(I46="",F46*$B$2/$B$1,F46)</f>
+        <v/>
+      </c>
+      <c r="K46" s="5">
+        <f>IF(I46="",H46*$B$2/$B$1,H46)</f>
+        <v/>
+      </c>
+      <c r="L46" s="5">
+        <f>IF(I46="",F46*$B$4/$B$3,F46)</f>
+        <v/>
+      </c>
+      <c r="M46" s="5">
+        <f>IF(I46="",H46*$B$4/$B$3,H46)</f>
+        <v/>
+      </c>
+      <c r="N46" s="5">
+        <f>IF(I46="",G46*$B$4/$B$3,G46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>39</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>프로피나정</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>648504140</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>신풍제약</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>728</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>4520</v>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>3290560</v>
+      </c>
+      <c r="I47">
+        <f>IF(G47&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J47" s="5">
+        <f>IF(I47="",F47*$B$2/$B$1,F47)</f>
+        <v/>
+      </c>
+      <c r="K47" s="5">
+        <f>IF(I47="",H47*$B$2/$B$1,H47)</f>
+        <v/>
+      </c>
+      <c r="L47" s="5">
+        <f>IF(I47="",F47*$B$4/$B$3,F47)</f>
+        <v/>
+      </c>
+      <c r="M47" s="5">
+        <f>IF(I47="",H47*$B$4/$B$3,H47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="5">
+        <f>IF(I47="",G47*$B$4/$B$3,G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>40</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>놀텍정10밀리그램</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>641702920</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>일양약품</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>1071</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>3072</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>3290112</v>
+      </c>
+      <c r="I48">
+        <f>IF(G48&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J48" s="5">
+        <f>IF(I48="",F48*$B$2/$B$1,F48)</f>
+        <v/>
+      </c>
+      <c r="K48" s="5">
+        <f>IF(I48="",H48*$B$2/$B$1,H48)</f>
+        <v/>
+      </c>
+      <c r="L48" s="5">
+        <f>IF(I48="",F48*$B$4/$B$3,F48)</f>
+        <v/>
+      </c>
+      <c r="M48" s="5">
+        <f>IF(I48="",H48*$B$4/$B$3,H48)</f>
+        <v/>
+      </c>
+      <c r="N48" s="5">
+        <f>IF(I48="",G48*$B$4/$B$3,G48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>41</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>뉴스타틴알정10밀리그램</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>647803940</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>삼진제약</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>585</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="G49" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>3175089</v>
+      </c>
+      <c r="I49">
+        <f>IF(G49&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J49" s="5">
+        <f>IF(I49="",F49*$B$2/$B$1,F49)</f>
+        <v/>
+      </c>
+      <c r="K49" s="5">
+        <f>IF(I49="",H49*$B$2/$B$1,H49)</f>
+        <v/>
+      </c>
+      <c r="L49" s="5">
+        <f>IF(I49="",F49*$B$4/$B$3,F49)</f>
+        <v/>
+      </c>
+      <c r="M49" s="5">
+        <f>IF(I49="",H49*$B$4/$B$3,H49)</f>
+        <v/>
+      </c>
+      <c r="N49" s="5">
+        <f>IF(I49="",G49*$B$4/$B$3,G49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>42</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>베아셉트정10밀리그램</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>694001100</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>대웅바이오</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v>2213</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>1427</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>3157951</v>
+      </c>
+      <c r="I50">
+        <f>IF(G50&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J50" s="5">
+        <f>IF(I50="",F50*$B$2/$B$1,F50)</f>
+        <v/>
+      </c>
+      <c r="K50" s="5">
+        <f>IF(I50="",H50*$B$2/$B$1,H50)</f>
+        <v/>
+      </c>
+      <c r="L50" s="5">
+        <f>IF(I50="",F50*$B$4/$B$3,F50)</f>
+        <v/>
+      </c>
+      <c r="M50" s="5">
+        <f>IF(I50="",H50*$B$4/$B$3,H50)</f>
+        <v/>
+      </c>
+      <c r="N50" s="5">
+        <f>IF(I50="",G50*$B$4/$B$3,G50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>43</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>시너지아정500mg</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2120857</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>1260</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>2441</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>3075660</v>
+      </c>
+      <c r="I51">
+        <f>IF(G51&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J51" s="5">
+        <f>IF(I51="",F51*$B$2/$B$1,F51)</f>
+        <v/>
+      </c>
+      <c r="K51" s="5">
+        <f>IF(I51="",H51*$B$2/$B$1,H51)</f>
+        <v/>
+      </c>
+      <c r="L51" s="5">
+        <f>IF(I51="",F51*$B$4/$B$3,F51)</f>
+        <v/>
+      </c>
+      <c r="M51" s="5">
+        <f>IF(I51="",H51*$B$4/$B$3,H51)</f>
+        <v/>
+      </c>
+      <c r="N51" s="5">
+        <f>IF(I51="",G51*$B$4/$B$3,G51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>44</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>리피로우정10밀리그램</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>643304610</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>(주)종근당</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>658</v>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>4599</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>3026142</v>
+      </c>
+      <c r="I52">
+        <f>IF(G52&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J52" s="5">
+        <f>IF(I52="",F52*$B$2/$B$1,F52)</f>
+        <v/>
+      </c>
+      <c r="K52" s="5">
+        <f>IF(I52="",H52*$B$2/$B$1,H52)</f>
+        <v/>
+      </c>
+      <c r="L52" s="5">
+        <f>IF(I52="",F52*$B$4/$B$3,F52)</f>
+        <v/>
+      </c>
+      <c r="M52" s="5">
+        <f>IF(I52="",H52*$B$4/$B$3,H52)</f>
+        <v/>
+      </c>
+      <c r="N52" s="5">
+        <f>IF(I52="",G52*$B$4/$B$3,G52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>45</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>비판티정2mg</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>648501460</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>신풍제약</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>355</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>8158</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="H53" s="5" t="n">
+        <v>2896090</v>
+      </c>
+      <c r="I53">
+        <f>IF(G53&lt;=$B$5,"일회성(환산제외)","")</f>
+        <v/>
+      </c>
+      <c r="J53" s="5">
+        <f>IF(I53="",F53*$B$2/$B$1,F53)</f>
+        <v/>
+      </c>
+      <c r="K53" s="5">
+        <f>IF(I53="",H53*$B$2/$B$1,H53)</f>
+        <v/>
+      </c>
+      <c r="L53" s="5">
+        <f>IF(I53="",F53*$B$4/$B$3,F53)</f>
+        <v/>
+      </c>
+      <c r="M53" s="5">
+        <f>IF(I53="",H53*$B$4/$B$3,H53)</f>
+        <v/>
+      </c>
+      <c r="N53" s="5">
+        <f>IF(I53="",G53*$B$4/$B$3,G53)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A8:N53"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1387,7 +4073,6 @@
       <c r="O14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2002,7 +4687,6 @@
           <t>2120438</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>0</t>
@@ -3318,7 +6002,6 @@
           <t>2120857</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>0</t>
@@ -3499,7 +6182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6242,7 +8925,6 @@
       <c r="O41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -6527,7 +9209,6 @@
           <t>2120761</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>0</t>
@@ -9534,7 +12215,6 @@
       <c r="O91" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">

</xml_diff>

<commit_message>
Multiply monthly projection columns by 2 via adjustable multiplier
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015f56A799NhnuL2TDwF4NVd
</commit_message>
<xml_diff>
--- a/조제내역_약가합계순.xlsx
+++ b/조제내역_약가합계순.xlsx
@@ -520,6 +520,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>곱하는 배수(한달 환산 열 전체)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>영업일은 일요일, 5/1, 5/5, 5/25(대체공휴일) 휴무로 가정한 값입니다. 실제 휴무일에 맞게 노란 칸(B3, B4)을 고치면 전체가 다시 계산됩니다.</t>
         </is>
       </c>
@@ -632,23 +642,23 @@
         <v/>
       </c>
       <c r="J9" s="5">
-        <f>IF(I9="",F9*$B$2/$B$1,F9)</f>
+        <f>(IF(I9="",F9*$B$2/$B$1,F9))*$B$6</f>
         <v/>
       </c>
       <c r="K9" s="5">
-        <f>IF(I9="",H9*$B$2/$B$1,H9)</f>
+        <f>(IF(I9="",H9*$B$2/$B$1,H9))*$B$6</f>
         <v/>
       </c>
       <c r="L9" s="5">
-        <f>IF(I9="",F9*$B$4/$B$3,F9)</f>
+        <f>(IF(I9="",F9*$B$4/$B$3,F9))*$B$6</f>
         <v/>
       </c>
       <c r="M9" s="5">
-        <f>IF(I9="",H9*$B$4/$B$3,H9)</f>
+        <f>(IF(I9="",H9*$B$4/$B$3,H9))*$B$6</f>
         <v/>
       </c>
       <c r="N9" s="5">
-        <f>IF(I9="",G9*$B$4/$B$3,G9)</f>
+        <f>(IF(I9="",G9*$B$4/$B$3,G9))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -688,23 +698,23 @@
         <v/>
       </c>
       <c r="J10" s="5">
-        <f>IF(I10="",F10*$B$2/$B$1,F10)</f>
+        <f>(IF(I10="",F10*$B$2/$B$1,F10))*$B$6</f>
         <v/>
       </c>
       <c r="K10" s="5">
-        <f>IF(I10="",H10*$B$2/$B$1,H10)</f>
+        <f>(IF(I10="",H10*$B$2/$B$1,H10))*$B$6</f>
         <v/>
       </c>
       <c r="L10" s="5">
-        <f>IF(I10="",F10*$B$4/$B$3,F10)</f>
+        <f>(IF(I10="",F10*$B$4/$B$3,F10))*$B$6</f>
         <v/>
       </c>
       <c r="M10" s="5">
-        <f>IF(I10="",H10*$B$4/$B$3,H10)</f>
+        <f>(IF(I10="",H10*$B$4/$B$3,H10))*$B$6</f>
         <v/>
       </c>
       <c r="N10" s="5">
-        <f>IF(I10="",G10*$B$4/$B$3,G10)</f>
+        <f>(IF(I10="",G10*$B$4/$B$3,G10))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -744,23 +754,23 @@
         <v/>
       </c>
       <c r="J11" s="5">
-        <f>IF(I11="",F11*$B$2/$B$1,F11)</f>
+        <f>(IF(I11="",F11*$B$2/$B$1,F11))*$B$6</f>
         <v/>
       </c>
       <c r="K11" s="5">
-        <f>IF(I11="",H11*$B$2/$B$1,H11)</f>
+        <f>(IF(I11="",H11*$B$2/$B$1,H11))*$B$6</f>
         <v/>
       </c>
       <c r="L11" s="5">
-        <f>IF(I11="",F11*$B$4/$B$3,F11)</f>
+        <f>(IF(I11="",F11*$B$4/$B$3,F11))*$B$6</f>
         <v/>
       </c>
       <c r="M11" s="5">
-        <f>IF(I11="",H11*$B$4/$B$3,H11)</f>
+        <f>(IF(I11="",H11*$B$4/$B$3,H11))*$B$6</f>
         <v/>
       </c>
       <c r="N11" s="5">
-        <f>IF(I11="",G11*$B$4/$B$3,G11)</f>
+        <f>(IF(I11="",G11*$B$4/$B$3,G11))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -800,23 +810,23 @@
         <v/>
       </c>
       <c r="J12" s="5">
-        <f>IF(I12="",F12*$B$2/$B$1,F12)</f>
+        <f>(IF(I12="",F12*$B$2/$B$1,F12))*$B$6</f>
         <v/>
       </c>
       <c r="K12" s="5">
-        <f>IF(I12="",H12*$B$2/$B$1,H12)</f>
+        <f>(IF(I12="",H12*$B$2/$B$1,H12))*$B$6</f>
         <v/>
       </c>
       <c r="L12" s="5">
-        <f>IF(I12="",F12*$B$4/$B$3,F12)</f>
+        <f>(IF(I12="",F12*$B$4/$B$3,F12))*$B$6</f>
         <v/>
       </c>
       <c r="M12" s="5">
-        <f>IF(I12="",H12*$B$4/$B$3,H12)</f>
+        <f>(IF(I12="",H12*$B$4/$B$3,H12))*$B$6</f>
         <v/>
       </c>
       <c r="N12" s="5">
-        <f>IF(I12="",G12*$B$4/$B$3,G12)</f>
+        <f>(IF(I12="",G12*$B$4/$B$3,G12))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -856,23 +866,23 @@
         <v/>
       </c>
       <c r="J13" s="5">
-        <f>IF(I13="",F13*$B$2/$B$1,F13)</f>
+        <f>(IF(I13="",F13*$B$2/$B$1,F13))*$B$6</f>
         <v/>
       </c>
       <c r="K13" s="5">
-        <f>IF(I13="",H13*$B$2/$B$1,H13)</f>
+        <f>(IF(I13="",H13*$B$2/$B$1,H13))*$B$6</f>
         <v/>
       </c>
       <c r="L13" s="5">
-        <f>IF(I13="",F13*$B$4/$B$3,F13)</f>
+        <f>(IF(I13="",F13*$B$4/$B$3,F13))*$B$6</f>
         <v/>
       </c>
       <c r="M13" s="5">
-        <f>IF(I13="",H13*$B$4/$B$3,H13)</f>
+        <f>(IF(I13="",H13*$B$4/$B$3,H13))*$B$6</f>
         <v/>
       </c>
       <c r="N13" s="5">
-        <f>IF(I13="",G13*$B$4/$B$3,G13)</f>
+        <f>(IF(I13="",G13*$B$4/$B$3,G13))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -912,23 +922,23 @@
         <v/>
       </c>
       <c r="J14" s="5">
-        <f>IF(I14="",F14*$B$2/$B$1,F14)</f>
+        <f>(IF(I14="",F14*$B$2/$B$1,F14))*$B$6</f>
         <v/>
       </c>
       <c r="K14" s="5">
-        <f>IF(I14="",H14*$B$2/$B$1,H14)</f>
+        <f>(IF(I14="",H14*$B$2/$B$1,H14))*$B$6</f>
         <v/>
       </c>
       <c r="L14" s="5">
-        <f>IF(I14="",F14*$B$4/$B$3,F14)</f>
+        <f>(IF(I14="",F14*$B$4/$B$3,F14))*$B$6</f>
         <v/>
       </c>
       <c r="M14" s="5">
-        <f>IF(I14="",H14*$B$4/$B$3,H14)</f>
+        <f>(IF(I14="",H14*$B$4/$B$3,H14))*$B$6</f>
         <v/>
       </c>
       <c r="N14" s="5">
-        <f>IF(I14="",G14*$B$4/$B$3,G14)</f>
+        <f>(IF(I14="",G14*$B$4/$B$3,G14))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -968,23 +978,23 @@
         <v/>
       </c>
       <c r="J15" s="5">
-        <f>IF(I15="",F15*$B$2/$B$1,F15)</f>
+        <f>(IF(I15="",F15*$B$2/$B$1,F15))*$B$6</f>
         <v/>
       </c>
       <c r="K15" s="5">
-        <f>IF(I15="",H15*$B$2/$B$1,H15)</f>
+        <f>(IF(I15="",H15*$B$2/$B$1,H15))*$B$6</f>
         <v/>
       </c>
       <c r="L15" s="5">
-        <f>IF(I15="",F15*$B$4/$B$3,F15)</f>
+        <f>(IF(I15="",F15*$B$4/$B$3,F15))*$B$6</f>
         <v/>
       </c>
       <c r="M15" s="5">
-        <f>IF(I15="",H15*$B$4/$B$3,H15)</f>
+        <f>(IF(I15="",H15*$B$4/$B$3,H15))*$B$6</f>
         <v/>
       </c>
       <c r="N15" s="5">
-        <f>IF(I15="",G15*$B$4/$B$3,G15)</f>
+        <f>(IF(I15="",G15*$B$4/$B$3,G15))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1024,23 +1034,23 @@
         <v/>
       </c>
       <c r="J16" s="5">
-        <f>IF(I16="",F16*$B$2/$B$1,F16)</f>
+        <f>(IF(I16="",F16*$B$2/$B$1,F16))*$B$6</f>
         <v/>
       </c>
       <c r="K16" s="5">
-        <f>IF(I16="",H16*$B$2/$B$1,H16)</f>
+        <f>(IF(I16="",H16*$B$2/$B$1,H16))*$B$6</f>
         <v/>
       </c>
       <c r="L16" s="5">
-        <f>IF(I16="",F16*$B$4/$B$3,F16)</f>
+        <f>(IF(I16="",F16*$B$4/$B$3,F16))*$B$6</f>
         <v/>
       </c>
       <c r="M16" s="5">
-        <f>IF(I16="",H16*$B$4/$B$3,H16)</f>
+        <f>(IF(I16="",H16*$B$4/$B$3,H16))*$B$6</f>
         <v/>
       </c>
       <c r="N16" s="5">
-        <f>IF(I16="",G16*$B$4/$B$3,G16)</f>
+        <f>(IF(I16="",G16*$B$4/$B$3,G16))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1080,23 +1090,23 @@
         <v/>
       </c>
       <c r="J17" s="5">
-        <f>IF(I17="",F17*$B$2/$B$1,F17)</f>
+        <f>(IF(I17="",F17*$B$2/$B$1,F17))*$B$6</f>
         <v/>
       </c>
       <c r="K17" s="5">
-        <f>IF(I17="",H17*$B$2/$B$1,H17)</f>
+        <f>(IF(I17="",H17*$B$2/$B$1,H17))*$B$6</f>
         <v/>
       </c>
       <c r="L17" s="5">
-        <f>IF(I17="",F17*$B$4/$B$3,F17)</f>
+        <f>(IF(I17="",F17*$B$4/$B$3,F17))*$B$6</f>
         <v/>
       </c>
       <c r="M17" s="5">
-        <f>IF(I17="",H17*$B$4/$B$3,H17)</f>
+        <f>(IF(I17="",H17*$B$4/$B$3,H17))*$B$6</f>
         <v/>
       </c>
       <c r="N17" s="5">
-        <f>IF(I17="",G17*$B$4/$B$3,G17)</f>
+        <f>(IF(I17="",G17*$B$4/$B$3,G17))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1136,23 +1146,23 @@
         <v/>
       </c>
       <c r="J18" s="5">
-        <f>IF(I18="",F18*$B$2/$B$1,F18)</f>
+        <f>(IF(I18="",F18*$B$2/$B$1,F18))*$B$6</f>
         <v/>
       </c>
       <c r="K18" s="5">
-        <f>IF(I18="",H18*$B$2/$B$1,H18)</f>
+        <f>(IF(I18="",H18*$B$2/$B$1,H18))*$B$6</f>
         <v/>
       </c>
       <c r="L18" s="5">
-        <f>IF(I18="",F18*$B$4/$B$3,F18)</f>
+        <f>(IF(I18="",F18*$B$4/$B$3,F18))*$B$6</f>
         <v/>
       </c>
       <c r="M18" s="5">
-        <f>IF(I18="",H18*$B$4/$B$3,H18)</f>
+        <f>(IF(I18="",H18*$B$4/$B$3,H18))*$B$6</f>
         <v/>
       </c>
       <c r="N18" s="5">
-        <f>IF(I18="",G18*$B$4/$B$3,G18)</f>
+        <f>(IF(I18="",G18*$B$4/$B$3,G18))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1192,23 +1202,23 @@
         <v/>
       </c>
       <c r="J19" s="5">
-        <f>IF(I19="",F19*$B$2/$B$1,F19)</f>
+        <f>(IF(I19="",F19*$B$2/$B$1,F19))*$B$6</f>
         <v/>
       </c>
       <c r="K19" s="5">
-        <f>IF(I19="",H19*$B$2/$B$1,H19)</f>
+        <f>(IF(I19="",H19*$B$2/$B$1,H19))*$B$6</f>
         <v/>
       </c>
       <c r="L19" s="5">
-        <f>IF(I19="",F19*$B$4/$B$3,F19)</f>
+        <f>(IF(I19="",F19*$B$4/$B$3,F19))*$B$6</f>
         <v/>
       </c>
       <c r="M19" s="5">
-        <f>IF(I19="",H19*$B$4/$B$3,H19)</f>
+        <f>(IF(I19="",H19*$B$4/$B$3,H19))*$B$6</f>
         <v/>
       </c>
       <c r="N19" s="5">
-        <f>IF(I19="",G19*$B$4/$B$3,G19)</f>
+        <f>(IF(I19="",G19*$B$4/$B$3,G19))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1248,23 +1258,23 @@
         <v/>
       </c>
       <c r="J20" s="5">
-        <f>IF(I20="",F20*$B$2/$B$1,F20)</f>
+        <f>(IF(I20="",F20*$B$2/$B$1,F20))*$B$6</f>
         <v/>
       </c>
       <c r="K20" s="5">
-        <f>IF(I20="",H20*$B$2/$B$1,H20)</f>
+        <f>(IF(I20="",H20*$B$2/$B$1,H20))*$B$6</f>
         <v/>
       </c>
       <c r="L20" s="5">
-        <f>IF(I20="",F20*$B$4/$B$3,F20)</f>
+        <f>(IF(I20="",F20*$B$4/$B$3,F20))*$B$6</f>
         <v/>
       </c>
       <c r="M20" s="5">
-        <f>IF(I20="",H20*$B$4/$B$3,H20)</f>
+        <f>(IF(I20="",H20*$B$4/$B$3,H20))*$B$6</f>
         <v/>
       </c>
       <c r="N20" s="5">
-        <f>IF(I20="",G20*$B$4/$B$3,G20)</f>
+        <f>(IF(I20="",G20*$B$4/$B$3,G20))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1304,23 +1314,23 @@
         <v/>
       </c>
       <c r="J21" s="5">
-        <f>IF(I21="",F21*$B$2/$B$1,F21)</f>
+        <f>(IF(I21="",F21*$B$2/$B$1,F21))*$B$6</f>
         <v/>
       </c>
       <c r="K21" s="5">
-        <f>IF(I21="",H21*$B$2/$B$1,H21)</f>
+        <f>(IF(I21="",H21*$B$2/$B$1,H21))*$B$6</f>
         <v/>
       </c>
       <c r="L21" s="5">
-        <f>IF(I21="",F21*$B$4/$B$3,F21)</f>
+        <f>(IF(I21="",F21*$B$4/$B$3,F21))*$B$6</f>
         <v/>
       </c>
       <c r="M21" s="5">
-        <f>IF(I21="",H21*$B$4/$B$3,H21)</f>
+        <f>(IF(I21="",H21*$B$4/$B$3,H21))*$B$6</f>
         <v/>
       </c>
       <c r="N21" s="5">
-        <f>IF(I21="",G21*$B$4/$B$3,G21)</f>
+        <f>(IF(I21="",G21*$B$4/$B$3,G21))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1360,23 +1370,23 @@
         <v/>
       </c>
       <c r="J22" s="5">
-        <f>IF(I22="",F22*$B$2/$B$1,F22)</f>
+        <f>(IF(I22="",F22*$B$2/$B$1,F22))*$B$6</f>
         <v/>
       </c>
       <c r="K22" s="5">
-        <f>IF(I22="",H22*$B$2/$B$1,H22)</f>
+        <f>(IF(I22="",H22*$B$2/$B$1,H22))*$B$6</f>
         <v/>
       </c>
       <c r="L22" s="5">
-        <f>IF(I22="",F22*$B$4/$B$3,F22)</f>
+        <f>(IF(I22="",F22*$B$4/$B$3,F22))*$B$6</f>
         <v/>
       </c>
       <c r="M22" s="5">
-        <f>IF(I22="",H22*$B$4/$B$3,H22)</f>
+        <f>(IF(I22="",H22*$B$4/$B$3,H22))*$B$6</f>
         <v/>
       </c>
       <c r="N22" s="5">
-        <f>IF(I22="",G22*$B$4/$B$3,G22)</f>
+        <f>(IF(I22="",G22*$B$4/$B$3,G22))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1416,23 +1426,23 @@
         <v/>
       </c>
       <c r="J23" s="5">
-        <f>IF(I23="",F23*$B$2/$B$1,F23)</f>
+        <f>(IF(I23="",F23*$B$2/$B$1,F23))*$B$6</f>
         <v/>
       </c>
       <c r="K23" s="5">
-        <f>IF(I23="",H23*$B$2/$B$1,H23)</f>
+        <f>(IF(I23="",H23*$B$2/$B$1,H23))*$B$6</f>
         <v/>
       </c>
       <c r="L23" s="5">
-        <f>IF(I23="",F23*$B$4/$B$3,F23)</f>
+        <f>(IF(I23="",F23*$B$4/$B$3,F23))*$B$6</f>
         <v/>
       </c>
       <c r="M23" s="5">
-        <f>IF(I23="",H23*$B$4/$B$3,H23)</f>
+        <f>(IF(I23="",H23*$B$4/$B$3,H23))*$B$6</f>
         <v/>
       </c>
       <c r="N23" s="5">
-        <f>IF(I23="",G23*$B$4/$B$3,G23)</f>
+        <f>(IF(I23="",G23*$B$4/$B$3,G23))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1472,23 +1482,23 @@
         <v/>
       </c>
       <c r="J24" s="5">
-        <f>IF(I24="",F24*$B$2/$B$1,F24)</f>
+        <f>(IF(I24="",F24*$B$2/$B$1,F24))*$B$6</f>
         <v/>
       </c>
       <c r="K24" s="5">
-        <f>IF(I24="",H24*$B$2/$B$1,H24)</f>
+        <f>(IF(I24="",H24*$B$2/$B$1,H24))*$B$6</f>
         <v/>
       </c>
       <c r="L24" s="5">
-        <f>IF(I24="",F24*$B$4/$B$3,F24)</f>
+        <f>(IF(I24="",F24*$B$4/$B$3,F24))*$B$6</f>
         <v/>
       </c>
       <c r="M24" s="5">
-        <f>IF(I24="",H24*$B$4/$B$3,H24)</f>
+        <f>(IF(I24="",H24*$B$4/$B$3,H24))*$B$6</f>
         <v/>
       </c>
       <c r="N24" s="5">
-        <f>IF(I24="",G24*$B$4/$B$3,G24)</f>
+        <f>(IF(I24="",G24*$B$4/$B$3,G24))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1528,23 +1538,23 @@
         <v/>
       </c>
       <c r="J25" s="5">
-        <f>IF(I25="",F25*$B$2/$B$1,F25)</f>
+        <f>(IF(I25="",F25*$B$2/$B$1,F25))*$B$6</f>
         <v/>
       </c>
       <c r="K25" s="5">
-        <f>IF(I25="",H25*$B$2/$B$1,H25)</f>
+        <f>(IF(I25="",H25*$B$2/$B$1,H25))*$B$6</f>
         <v/>
       </c>
       <c r="L25" s="5">
-        <f>IF(I25="",F25*$B$4/$B$3,F25)</f>
+        <f>(IF(I25="",F25*$B$4/$B$3,F25))*$B$6</f>
         <v/>
       </c>
       <c r="M25" s="5">
-        <f>IF(I25="",H25*$B$4/$B$3,H25)</f>
+        <f>(IF(I25="",H25*$B$4/$B$3,H25))*$B$6</f>
         <v/>
       </c>
       <c r="N25" s="5">
-        <f>IF(I25="",G25*$B$4/$B$3,G25)</f>
+        <f>(IF(I25="",G25*$B$4/$B$3,G25))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1584,23 +1594,23 @@
         <v/>
       </c>
       <c r="J26" s="5">
-        <f>IF(I26="",F26*$B$2/$B$1,F26)</f>
+        <f>(IF(I26="",F26*$B$2/$B$1,F26))*$B$6</f>
         <v/>
       </c>
       <c r="K26" s="5">
-        <f>IF(I26="",H26*$B$2/$B$1,H26)</f>
+        <f>(IF(I26="",H26*$B$2/$B$1,H26))*$B$6</f>
         <v/>
       </c>
       <c r="L26" s="5">
-        <f>IF(I26="",F26*$B$4/$B$3,F26)</f>
+        <f>(IF(I26="",F26*$B$4/$B$3,F26))*$B$6</f>
         <v/>
       </c>
       <c r="M26" s="5">
-        <f>IF(I26="",H26*$B$4/$B$3,H26)</f>
+        <f>(IF(I26="",H26*$B$4/$B$3,H26))*$B$6</f>
         <v/>
       </c>
       <c r="N26" s="5">
-        <f>IF(I26="",G26*$B$4/$B$3,G26)</f>
+        <f>(IF(I26="",G26*$B$4/$B$3,G26))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1640,23 +1650,23 @@
         <v/>
       </c>
       <c r="J27" s="5">
-        <f>IF(I27="",F27*$B$2/$B$1,F27)</f>
+        <f>(IF(I27="",F27*$B$2/$B$1,F27))*$B$6</f>
         <v/>
       </c>
       <c r="K27" s="5">
-        <f>IF(I27="",H27*$B$2/$B$1,H27)</f>
+        <f>(IF(I27="",H27*$B$2/$B$1,H27))*$B$6</f>
         <v/>
       </c>
       <c r="L27" s="5">
-        <f>IF(I27="",F27*$B$4/$B$3,F27)</f>
+        <f>(IF(I27="",F27*$B$4/$B$3,F27))*$B$6</f>
         <v/>
       </c>
       <c r="M27" s="5">
-        <f>IF(I27="",H27*$B$4/$B$3,H27)</f>
+        <f>(IF(I27="",H27*$B$4/$B$3,H27))*$B$6</f>
         <v/>
       </c>
       <c r="N27" s="5">
-        <f>IF(I27="",G27*$B$4/$B$3,G27)</f>
+        <f>(IF(I27="",G27*$B$4/$B$3,G27))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1696,23 +1706,23 @@
         <v/>
       </c>
       <c r="J28" s="5">
-        <f>IF(I28="",F28*$B$2/$B$1,F28)</f>
+        <f>(IF(I28="",F28*$B$2/$B$1,F28))*$B$6</f>
         <v/>
       </c>
       <c r="K28" s="5">
-        <f>IF(I28="",H28*$B$2/$B$1,H28)</f>
+        <f>(IF(I28="",H28*$B$2/$B$1,H28))*$B$6</f>
         <v/>
       </c>
       <c r="L28" s="5">
-        <f>IF(I28="",F28*$B$4/$B$3,F28)</f>
+        <f>(IF(I28="",F28*$B$4/$B$3,F28))*$B$6</f>
         <v/>
       </c>
       <c r="M28" s="5">
-        <f>IF(I28="",H28*$B$4/$B$3,H28)</f>
+        <f>(IF(I28="",H28*$B$4/$B$3,H28))*$B$6</f>
         <v/>
       </c>
       <c r="N28" s="5">
-        <f>IF(I28="",G28*$B$4/$B$3,G28)</f>
+        <f>(IF(I28="",G28*$B$4/$B$3,G28))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1752,23 +1762,23 @@
         <v/>
       </c>
       <c r="J29" s="5">
-        <f>IF(I29="",F29*$B$2/$B$1,F29)</f>
+        <f>(IF(I29="",F29*$B$2/$B$1,F29))*$B$6</f>
         <v/>
       </c>
       <c r="K29" s="5">
-        <f>IF(I29="",H29*$B$2/$B$1,H29)</f>
+        <f>(IF(I29="",H29*$B$2/$B$1,H29))*$B$6</f>
         <v/>
       </c>
       <c r="L29" s="5">
-        <f>IF(I29="",F29*$B$4/$B$3,F29)</f>
+        <f>(IF(I29="",F29*$B$4/$B$3,F29))*$B$6</f>
         <v/>
       </c>
       <c r="M29" s="5">
-        <f>IF(I29="",H29*$B$4/$B$3,H29)</f>
+        <f>(IF(I29="",H29*$B$4/$B$3,H29))*$B$6</f>
         <v/>
       </c>
       <c r="N29" s="5">
-        <f>IF(I29="",G29*$B$4/$B$3,G29)</f>
+        <f>(IF(I29="",G29*$B$4/$B$3,G29))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1803,23 +1813,23 @@
         <v/>
       </c>
       <c r="J30" s="5">
-        <f>IF(I30="",F30*$B$2/$B$1,F30)</f>
+        <f>(IF(I30="",F30*$B$2/$B$1,F30))*$B$6</f>
         <v/>
       </c>
       <c r="K30" s="5">
-        <f>IF(I30="",H30*$B$2/$B$1,H30)</f>
+        <f>(IF(I30="",H30*$B$2/$B$1,H30))*$B$6</f>
         <v/>
       </c>
       <c r="L30" s="5">
-        <f>IF(I30="",F30*$B$4/$B$3,F30)</f>
+        <f>(IF(I30="",F30*$B$4/$B$3,F30))*$B$6</f>
         <v/>
       </c>
       <c r="M30" s="5">
-        <f>IF(I30="",H30*$B$4/$B$3,H30)</f>
+        <f>(IF(I30="",H30*$B$4/$B$3,H30))*$B$6</f>
         <v/>
       </c>
       <c r="N30" s="5">
-        <f>IF(I30="",G30*$B$4/$B$3,G30)</f>
+        <f>(IF(I30="",G30*$B$4/$B$3,G30))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1859,23 +1869,23 @@
         <v/>
       </c>
       <c r="J31" s="5">
-        <f>IF(I31="",F31*$B$2/$B$1,F31)</f>
+        <f>(IF(I31="",F31*$B$2/$B$1,F31))*$B$6</f>
         <v/>
       </c>
       <c r="K31" s="5">
-        <f>IF(I31="",H31*$B$2/$B$1,H31)</f>
+        <f>(IF(I31="",H31*$B$2/$B$1,H31))*$B$6</f>
         <v/>
       </c>
       <c r="L31" s="5">
-        <f>IF(I31="",F31*$B$4/$B$3,F31)</f>
+        <f>(IF(I31="",F31*$B$4/$B$3,F31))*$B$6</f>
         <v/>
       </c>
       <c r="M31" s="5">
-        <f>IF(I31="",H31*$B$4/$B$3,H31)</f>
+        <f>(IF(I31="",H31*$B$4/$B$3,H31))*$B$6</f>
         <v/>
       </c>
       <c r="N31" s="5">
-        <f>IF(I31="",G31*$B$4/$B$3,G31)</f>
+        <f>(IF(I31="",G31*$B$4/$B$3,G31))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1915,23 +1925,23 @@
         <v/>
       </c>
       <c r="J32" s="5">
-        <f>IF(I32="",F32*$B$2/$B$1,F32)</f>
+        <f>(IF(I32="",F32*$B$2/$B$1,F32))*$B$6</f>
         <v/>
       </c>
       <c r="K32" s="5">
-        <f>IF(I32="",H32*$B$2/$B$1,H32)</f>
+        <f>(IF(I32="",H32*$B$2/$B$1,H32))*$B$6</f>
         <v/>
       </c>
       <c r="L32" s="5">
-        <f>IF(I32="",F32*$B$4/$B$3,F32)</f>
+        <f>(IF(I32="",F32*$B$4/$B$3,F32))*$B$6</f>
         <v/>
       </c>
       <c r="M32" s="5">
-        <f>IF(I32="",H32*$B$4/$B$3,H32)</f>
+        <f>(IF(I32="",H32*$B$4/$B$3,H32))*$B$6</f>
         <v/>
       </c>
       <c r="N32" s="5">
-        <f>IF(I32="",G32*$B$4/$B$3,G32)</f>
+        <f>(IF(I32="",G32*$B$4/$B$3,G32))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -1971,23 +1981,23 @@
         <v/>
       </c>
       <c r="J33" s="5">
-        <f>IF(I33="",F33*$B$2/$B$1,F33)</f>
+        <f>(IF(I33="",F33*$B$2/$B$1,F33))*$B$6</f>
         <v/>
       </c>
       <c r="K33" s="5">
-        <f>IF(I33="",H33*$B$2/$B$1,H33)</f>
+        <f>(IF(I33="",H33*$B$2/$B$1,H33))*$B$6</f>
         <v/>
       </c>
       <c r="L33" s="5">
-        <f>IF(I33="",F33*$B$4/$B$3,F33)</f>
+        <f>(IF(I33="",F33*$B$4/$B$3,F33))*$B$6</f>
         <v/>
       </c>
       <c r="M33" s="5">
-        <f>IF(I33="",H33*$B$4/$B$3,H33)</f>
+        <f>(IF(I33="",H33*$B$4/$B$3,H33))*$B$6</f>
         <v/>
       </c>
       <c r="N33" s="5">
-        <f>IF(I33="",G33*$B$4/$B$3,G33)</f>
+        <f>(IF(I33="",G33*$B$4/$B$3,G33))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2027,23 +2037,23 @@
         <v/>
       </c>
       <c r="J34" s="5">
-        <f>IF(I34="",F34*$B$2/$B$1,F34)</f>
+        <f>(IF(I34="",F34*$B$2/$B$1,F34))*$B$6</f>
         <v/>
       </c>
       <c r="K34" s="5">
-        <f>IF(I34="",H34*$B$2/$B$1,H34)</f>
+        <f>(IF(I34="",H34*$B$2/$B$1,H34))*$B$6</f>
         <v/>
       </c>
       <c r="L34" s="5">
-        <f>IF(I34="",F34*$B$4/$B$3,F34)</f>
+        <f>(IF(I34="",F34*$B$4/$B$3,F34))*$B$6</f>
         <v/>
       </c>
       <c r="M34" s="5">
-        <f>IF(I34="",H34*$B$4/$B$3,H34)</f>
+        <f>(IF(I34="",H34*$B$4/$B$3,H34))*$B$6</f>
         <v/>
       </c>
       <c r="N34" s="5">
-        <f>IF(I34="",G34*$B$4/$B$3,G34)</f>
+        <f>(IF(I34="",G34*$B$4/$B$3,G34))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2083,23 +2093,23 @@
         <v/>
       </c>
       <c r="J35" s="5">
-        <f>IF(I35="",F35*$B$2/$B$1,F35)</f>
+        <f>(IF(I35="",F35*$B$2/$B$1,F35))*$B$6</f>
         <v/>
       </c>
       <c r="K35" s="5">
-        <f>IF(I35="",H35*$B$2/$B$1,H35)</f>
+        <f>(IF(I35="",H35*$B$2/$B$1,H35))*$B$6</f>
         <v/>
       </c>
       <c r="L35" s="5">
-        <f>IF(I35="",F35*$B$4/$B$3,F35)</f>
+        <f>(IF(I35="",F35*$B$4/$B$3,F35))*$B$6</f>
         <v/>
       </c>
       <c r="M35" s="5">
-        <f>IF(I35="",H35*$B$4/$B$3,H35)</f>
+        <f>(IF(I35="",H35*$B$4/$B$3,H35))*$B$6</f>
         <v/>
       </c>
       <c r="N35" s="5">
-        <f>IF(I35="",G35*$B$4/$B$3,G35)</f>
+        <f>(IF(I35="",G35*$B$4/$B$3,G35))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2139,23 +2149,23 @@
         <v/>
       </c>
       <c r="J36" s="5">
-        <f>IF(I36="",F36*$B$2/$B$1,F36)</f>
+        <f>(IF(I36="",F36*$B$2/$B$1,F36))*$B$6</f>
         <v/>
       </c>
       <c r="K36" s="5">
-        <f>IF(I36="",H36*$B$2/$B$1,H36)</f>
+        <f>(IF(I36="",H36*$B$2/$B$1,H36))*$B$6</f>
         <v/>
       </c>
       <c r="L36" s="5">
-        <f>IF(I36="",F36*$B$4/$B$3,F36)</f>
+        <f>(IF(I36="",F36*$B$4/$B$3,F36))*$B$6</f>
         <v/>
       </c>
       <c r="M36" s="5">
-        <f>IF(I36="",H36*$B$4/$B$3,H36)</f>
+        <f>(IF(I36="",H36*$B$4/$B$3,H36))*$B$6</f>
         <v/>
       </c>
       <c r="N36" s="5">
-        <f>IF(I36="",G36*$B$4/$B$3,G36)</f>
+        <f>(IF(I36="",G36*$B$4/$B$3,G36))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2195,23 +2205,23 @@
         <v/>
       </c>
       <c r="J37" s="5">
-        <f>IF(I37="",F37*$B$2/$B$1,F37)</f>
+        <f>(IF(I37="",F37*$B$2/$B$1,F37))*$B$6</f>
         <v/>
       </c>
       <c r="K37" s="5">
-        <f>IF(I37="",H37*$B$2/$B$1,H37)</f>
+        <f>(IF(I37="",H37*$B$2/$B$1,H37))*$B$6</f>
         <v/>
       </c>
       <c r="L37" s="5">
-        <f>IF(I37="",F37*$B$4/$B$3,F37)</f>
+        <f>(IF(I37="",F37*$B$4/$B$3,F37))*$B$6</f>
         <v/>
       </c>
       <c r="M37" s="5">
-        <f>IF(I37="",H37*$B$4/$B$3,H37)</f>
+        <f>(IF(I37="",H37*$B$4/$B$3,H37))*$B$6</f>
         <v/>
       </c>
       <c r="N37" s="5">
-        <f>IF(I37="",G37*$B$4/$B$3,G37)</f>
+        <f>(IF(I37="",G37*$B$4/$B$3,G37))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2251,23 +2261,23 @@
         <v/>
       </c>
       <c r="J38" s="5">
-        <f>IF(I38="",F38*$B$2/$B$1,F38)</f>
+        <f>(IF(I38="",F38*$B$2/$B$1,F38))*$B$6</f>
         <v/>
       </c>
       <c r="K38" s="5">
-        <f>IF(I38="",H38*$B$2/$B$1,H38)</f>
+        <f>(IF(I38="",H38*$B$2/$B$1,H38))*$B$6</f>
         <v/>
       </c>
       <c r="L38" s="5">
-        <f>IF(I38="",F38*$B$4/$B$3,F38)</f>
+        <f>(IF(I38="",F38*$B$4/$B$3,F38))*$B$6</f>
         <v/>
       </c>
       <c r="M38" s="5">
-        <f>IF(I38="",H38*$B$4/$B$3,H38)</f>
+        <f>(IF(I38="",H38*$B$4/$B$3,H38))*$B$6</f>
         <v/>
       </c>
       <c r="N38" s="5">
-        <f>IF(I38="",G38*$B$4/$B$3,G38)</f>
+        <f>(IF(I38="",G38*$B$4/$B$3,G38))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2307,23 +2317,23 @@
         <v/>
       </c>
       <c r="J39" s="5">
-        <f>IF(I39="",F39*$B$2/$B$1,F39)</f>
+        <f>(IF(I39="",F39*$B$2/$B$1,F39))*$B$6</f>
         <v/>
       </c>
       <c r="K39" s="5">
-        <f>IF(I39="",H39*$B$2/$B$1,H39)</f>
+        <f>(IF(I39="",H39*$B$2/$B$1,H39))*$B$6</f>
         <v/>
       </c>
       <c r="L39" s="5">
-        <f>IF(I39="",F39*$B$4/$B$3,F39)</f>
+        <f>(IF(I39="",F39*$B$4/$B$3,F39))*$B$6</f>
         <v/>
       </c>
       <c r="M39" s="5">
-        <f>IF(I39="",H39*$B$4/$B$3,H39)</f>
+        <f>(IF(I39="",H39*$B$4/$B$3,H39))*$B$6</f>
         <v/>
       </c>
       <c r="N39" s="5">
-        <f>IF(I39="",G39*$B$4/$B$3,G39)</f>
+        <f>(IF(I39="",G39*$B$4/$B$3,G39))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2363,23 +2373,23 @@
         <v/>
       </c>
       <c r="J40" s="5">
-        <f>IF(I40="",F40*$B$2/$B$1,F40)</f>
+        <f>(IF(I40="",F40*$B$2/$B$1,F40))*$B$6</f>
         <v/>
       </c>
       <c r="K40" s="5">
-        <f>IF(I40="",H40*$B$2/$B$1,H40)</f>
+        <f>(IF(I40="",H40*$B$2/$B$1,H40))*$B$6</f>
         <v/>
       </c>
       <c r="L40" s="5">
-        <f>IF(I40="",F40*$B$4/$B$3,F40)</f>
+        <f>(IF(I40="",F40*$B$4/$B$3,F40))*$B$6</f>
         <v/>
       </c>
       <c r="M40" s="5">
-        <f>IF(I40="",H40*$B$4/$B$3,H40)</f>
+        <f>(IF(I40="",H40*$B$4/$B$3,H40))*$B$6</f>
         <v/>
       </c>
       <c r="N40" s="5">
-        <f>IF(I40="",G40*$B$4/$B$3,G40)</f>
+        <f>(IF(I40="",G40*$B$4/$B$3,G40))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2419,23 +2429,23 @@
         <v/>
       </c>
       <c r="J41" s="5">
-        <f>IF(I41="",F41*$B$2/$B$1,F41)</f>
+        <f>(IF(I41="",F41*$B$2/$B$1,F41))*$B$6</f>
         <v/>
       </c>
       <c r="K41" s="5">
-        <f>IF(I41="",H41*$B$2/$B$1,H41)</f>
+        <f>(IF(I41="",H41*$B$2/$B$1,H41))*$B$6</f>
         <v/>
       </c>
       <c r="L41" s="5">
-        <f>IF(I41="",F41*$B$4/$B$3,F41)</f>
+        <f>(IF(I41="",F41*$B$4/$B$3,F41))*$B$6</f>
         <v/>
       </c>
       <c r="M41" s="5">
-        <f>IF(I41="",H41*$B$4/$B$3,H41)</f>
+        <f>(IF(I41="",H41*$B$4/$B$3,H41))*$B$6</f>
         <v/>
       </c>
       <c r="N41" s="5">
-        <f>IF(I41="",G41*$B$4/$B$3,G41)</f>
+        <f>(IF(I41="",G41*$B$4/$B$3,G41))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2475,23 +2485,23 @@
         <v/>
       </c>
       <c r="J42" s="5">
-        <f>IF(I42="",F42*$B$2/$B$1,F42)</f>
+        <f>(IF(I42="",F42*$B$2/$B$1,F42))*$B$6</f>
         <v/>
       </c>
       <c r="K42" s="5">
-        <f>IF(I42="",H42*$B$2/$B$1,H42)</f>
+        <f>(IF(I42="",H42*$B$2/$B$1,H42))*$B$6</f>
         <v/>
       </c>
       <c r="L42" s="5">
-        <f>IF(I42="",F42*$B$4/$B$3,F42)</f>
+        <f>(IF(I42="",F42*$B$4/$B$3,F42))*$B$6</f>
         <v/>
       </c>
       <c r="M42" s="5">
-        <f>IF(I42="",H42*$B$4/$B$3,H42)</f>
+        <f>(IF(I42="",H42*$B$4/$B$3,H42))*$B$6</f>
         <v/>
       </c>
       <c r="N42" s="5">
-        <f>IF(I42="",G42*$B$4/$B$3,G42)</f>
+        <f>(IF(I42="",G42*$B$4/$B$3,G42))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2531,23 +2541,23 @@
         <v/>
       </c>
       <c r="J43" s="5">
-        <f>IF(I43="",F43*$B$2/$B$1,F43)</f>
+        <f>(IF(I43="",F43*$B$2/$B$1,F43))*$B$6</f>
         <v/>
       </c>
       <c r="K43" s="5">
-        <f>IF(I43="",H43*$B$2/$B$1,H43)</f>
+        <f>(IF(I43="",H43*$B$2/$B$1,H43))*$B$6</f>
         <v/>
       </c>
       <c r="L43" s="5">
-        <f>IF(I43="",F43*$B$4/$B$3,F43)</f>
+        <f>(IF(I43="",F43*$B$4/$B$3,F43))*$B$6</f>
         <v/>
       </c>
       <c r="M43" s="5">
-        <f>IF(I43="",H43*$B$4/$B$3,H43)</f>
+        <f>(IF(I43="",H43*$B$4/$B$3,H43))*$B$6</f>
         <v/>
       </c>
       <c r="N43" s="5">
-        <f>IF(I43="",G43*$B$4/$B$3,G43)</f>
+        <f>(IF(I43="",G43*$B$4/$B$3,G43))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2587,23 +2597,23 @@
         <v/>
       </c>
       <c r="J44" s="5">
-        <f>IF(I44="",F44*$B$2/$B$1,F44)</f>
+        <f>(IF(I44="",F44*$B$2/$B$1,F44))*$B$6</f>
         <v/>
       </c>
       <c r="K44" s="5">
-        <f>IF(I44="",H44*$B$2/$B$1,H44)</f>
+        <f>(IF(I44="",H44*$B$2/$B$1,H44))*$B$6</f>
         <v/>
       </c>
       <c r="L44" s="5">
-        <f>IF(I44="",F44*$B$4/$B$3,F44)</f>
+        <f>(IF(I44="",F44*$B$4/$B$3,F44))*$B$6</f>
         <v/>
       </c>
       <c r="M44" s="5">
-        <f>IF(I44="",H44*$B$4/$B$3,H44)</f>
+        <f>(IF(I44="",H44*$B$4/$B$3,H44))*$B$6</f>
         <v/>
       </c>
       <c r="N44" s="5">
-        <f>IF(I44="",G44*$B$4/$B$3,G44)</f>
+        <f>(IF(I44="",G44*$B$4/$B$3,G44))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2643,23 +2653,23 @@
         <v/>
       </c>
       <c r="J45" s="5">
-        <f>IF(I45="",F45*$B$2/$B$1,F45)</f>
+        <f>(IF(I45="",F45*$B$2/$B$1,F45))*$B$6</f>
         <v/>
       </c>
       <c r="K45" s="5">
-        <f>IF(I45="",H45*$B$2/$B$1,H45)</f>
+        <f>(IF(I45="",H45*$B$2/$B$1,H45))*$B$6</f>
         <v/>
       </c>
       <c r="L45" s="5">
-        <f>IF(I45="",F45*$B$4/$B$3,F45)</f>
+        <f>(IF(I45="",F45*$B$4/$B$3,F45))*$B$6</f>
         <v/>
       </c>
       <c r="M45" s="5">
-        <f>IF(I45="",H45*$B$4/$B$3,H45)</f>
+        <f>(IF(I45="",H45*$B$4/$B$3,H45))*$B$6</f>
         <v/>
       </c>
       <c r="N45" s="5">
-        <f>IF(I45="",G45*$B$4/$B$3,G45)</f>
+        <f>(IF(I45="",G45*$B$4/$B$3,G45))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2699,23 +2709,23 @@
         <v/>
       </c>
       <c r="J46" s="5">
-        <f>IF(I46="",F46*$B$2/$B$1,F46)</f>
+        <f>(IF(I46="",F46*$B$2/$B$1,F46))*$B$6</f>
         <v/>
       </c>
       <c r="K46" s="5">
-        <f>IF(I46="",H46*$B$2/$B$1,H46)</f>
+        <f>(IF(I46="",H46*$B$2/$B$1,H46))*$B$6</f>
         <v/>
       </c>
       <c r="L46" s="5">
-        <f>IF(I46="",F46*$B$4/$B$3,F46)</f>
+        <f>(IF(I46="",F46*$B$4/$B$3,F46))*$B$6</f>
         <v/>
       </c>
       <c r="M46" s="5">
-        <f>IF(I46="",H46*$B$4/$B$3,H46)</f>
+        <f>(IF(I46="",H46*$B$4/$B$3,H46))*$B$6</f>
         <v/>
       </c>
       <c r="N46" s="5">
-        <f>IF(I46="",G46*$B$4/$B$3,G46)</f>
+        <f>(IF(I46="",G46*$B$4/$B$3,G46))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2755,23 +2765,23 @@
         <v/>
       </c>
       <c r="J47" s="5">
-        <f>IF(I47="",F47*$B$2/$B$1,F47)</f>
+        <f>(IF(I47="",F47*$B$2/$B$1,F47))*$B$6</f>
         <v/>
       </c>
       <c r="K47" s="5">
-        <f>IF(I47="",H47*$B$2/$B$1,H47)</f>
+        <f>(IF(I47="",H47*$B$2/$B$1,H47))*$B$6</f>
         <v/>
       </c>
       <c r="L47" s="5">
-        <f>IF(I47="",F47*$B$4/$B$3,F47)</f>
+        <f>(IF(I47="",F47*$B$4/$B$3,F47))*$B$6</f>
         <v/>
       </c>
       <c r="M47" s="5">
-        <f>IF(I47="",H47*$B$4/$B$3,H47)</f>
+        <f>(IF(I47="",H47*$B$4/$B$3,H47))*$B$6</f>
         <v/>
       </c>
       <c r="N47" s="5">
-        <f>IF(I47="",G47*$B$4/$B$3,G47)</f>
+        <f>(IF(I47="",G47*$B$4/$B$3,G47))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2811,23 +2821,23 @@
         <v/>
       </c>
       <c r="J48" s="5">
-        <f>IF(I48="",F48*$B$2/$B$1,F48)</f>
+        <f>(IF(I48="",F48*$B$2/$B$1,F48))*$B$6</f>
         <v/>
       </c>
       <c r="K48" s="5">
-        <f>IF(I48="",H48*$B$2/$B$1,H48)</f>
+        <f>(IF(I48="",H48*$B$2/$B$1,H48))*$B$6</f>
         <v/>
       </c>
       <c r="L48" s="5">
-        <f>IF(I48="",F48*$B$4/$B$3,F48)</f>
+        <f>(IF(I48="",F48*$B$4/$B$3,F48))*$B$6</f>
         <v/>
       </c>
       <c r="M48" s="5">
-        <f>IF(I48="",H48*$B$4/$B$3,H48)</f>
+        <f>(IF(I48="",H48*$B$4/$B$3,H48))*$B$6</f>
         <v/>
       </c>
       <c r="N48" s="5">
-        <f>IF(I48="",G48*$B$4/$B$3,G48)</f>
+        <f>(IF(I48="",G48*$B$4/$B$3,G48))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2867,23 +2877,23 @@
         <v/>
       </c>
       <c r="J49" s="5">
-        <f>IF(I49="",F49*$B$2/$B$1,F49)</f>
+        <f>(IF(I49="",F49*$B$2/$B$1,F49))*$B$6</f>
         <v/>
       </c>
       <c r="K49" s="5">
-        <f>IF(I49="",H49*$B$2/$B$1,H49)</f>
+        <f>(IF(I49="",H49*$B$2/$B$1,H49))*$B$6</f>
         <v/>
       </c>
       <c r="L49" s="5">
-        <f>IF(I49="",F49*$B$4/$B$3,F49)</f>
+        <f>(IF(I49="",F49*$B$4/$B$3,F49))*$B$6</f>
         <v/>
       </c>
       <c r="M49" s="5">
-        <f>IF(I49="",H49*$B$4/$B$3,H49)</f>
+        <f>(IF(I49="",H49*$B$4/$B$3,H49))*$B$6</f>
         <v/>
       </c>
       <c r="N49" s="5">
-        <f>IF(I49="",G49*$B$4/$B$3,G49)</f>
+        <f>(IF(I49="",G49*$B$4/$B$3,G49))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2923,23 +2933,23 @@
         <v/>
       </c>
       <c r="J50" s="5">
-        <f>IF(I50="",F50*$B$2/$B$1,F50)</f>
+        <f>(IF(I50="",F50*$B$2/$B$1,F50))*$B$6</f>
         <v/>
       </c>
       <c r="K50" s="5">
-        <f>IF(I50="",H50*$B$2/$B$1,H50)</f>
+        <f>(IF(I50="",H50*$B$2/$B$1,H50))*$B$6</f>
         <v/>
       </c>
       <c r="L50" s="5">
-        <f>IF(I50="",F50*$B$4/$B$3,F50)</f>
+        <f>(IF(I50="",F50*$B$4/$B$3,F50))*$B$6</f>
         <v/>
       </c>
       <c r="M50" s="5">
-        <f>IF(I50="",H50*$B$4/$B$3,H50)</f>
+        <f>(IF(I50="",H50*$B$4/$B$3,H50))*$B$6</f>
         <v/>
       </c>
       <c r="N50" s="5">
-        <f>IF(I50="",G50*$B$4/$B$3,G50)</f>
+        <f>(IF(I50="",G50*$B$4/$B$3,G50))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -2974,23 +2984,23 @@
         <v/>
       </c>
       <c r="J51" s="5">
-        <f>IF(I51="",F51*$B$2/$B$1,F51)</f>
+        <f>(IF(I51="",F51*$B$2/$B$1,F51))*$B$6</f>
         <v/>
       </c>
       <c r="K51" s="5">
-        <f>IF(I51="",H51*$B$2/$B$1,H51)</f>
+        <f>(IF(I51="",H51*$B$2/$B$1,H51))*$B$6</f>
         <v/>
       </c>
       <c r="L51" s="5">
-        <f>IF(I51="",F51*$B$4/$B$3,F51)</f>
+        <f>(IF(I51="",F51*$B$4/$B$3,F51))*$B$6</f>
         <v/>
       </c>
       <c r="M51" s="5">
-        <f>IF(I51="",H51*$B$4/$B$3,H51)</f>
+        <f>(IF(I51="",H51*$B$4/$B$3,H51))*$B$6</f>
         <v/>
       </c>
       <c r="N51" s="5">
-        <f>IF(I51="",G51*$B$4/$B$3,G51)</f>
+        <f>(IF(I51="",G51*$B$4/$B$3,G51))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -3030,23 +3040,23 @@
         <v/>
       </c>
       <c r="J52" s="5">
-        <f>IF(I52="",F52*$B$2/$B$1,F52)</f>
+        <f>(IF(I52="",F52*$B$2/$B$1,F52))*$B$6</f>
         <v/>
       </c>
       <c r="K52" s="5">
-        <f>IF(I52="",H52*$B$2/$B$1,H52)</f>
+        <f>(IF(I52="",H52*$B$2/$B$1,H52))*$B$6</f>
         <v/>
       </c>
       <c r="L52" s="5">
-        <f>IF(I52="",F52*$B$4/$B$3,F52)</f>
+        <f>(IF(I52="",F52*$B$4/$B$3,F52))*$B$6</f>
         <v/>
       </c>
       <c r="M52" s="5">
-        <f>IF(I52="",H52*$B$4/$B$3,H52)</f>
+        <f>(IF(I52="",H52*$B$4/$B$3,H52))*$B$6</f>
         <v/>
       </c>
       <c r="N52" s="5">
-        <f>IF(I52="",G52*$B$4/$B$3,G52)</f>
+        <f>(IF(I52="",G52*$B$4/$B$3,G52))*$B$6</f>
         <v/>
       </c>
     </row>
@@ -3086,23 +3096,23 @@
         <v/>
       </c>
       <c r="J53" s="5">
-        <f>IF(I53="",F53*$B$2/$B$1,F53)</f>
+        <f>(IF(I53="",F53*$B$2/$B$1,F53))*$B$6</f>
         <v/>
       </c>
       <c r="K53" s="5">
-        <f>IF(I53="",H53*$B$2/$B$1,H53)</f>
+        <f>(IF(I53="",H53*$B$2/$B$1,H53))*$B$6</f>
         <v/>
       </c>
       <c r="L53" s="5">
-        <f>IF(I53="",F53*$B$4/$B$3,F53)</f>
+        <f>(IF(I53="",F53*$B$4/$B$3,F53))*$B$6</f>
         <v/>
       </c>
       <c r="M53" s="5">
-        <f>IF(I53="",H53*$B$4/$B$3,H53)</f>
+        <f>(IF(I53="",H53*$B$4/$B$3,H53))*$B$6</f>
         <v/>
       </c>
       <c r="N53" s="5">
-        <f>IF(I53="",G53*$B$4/$B$3,G53)</f>
+        <f>(IF(I53="",G53*$B$4/$B$3,G53))*$B$6</f>
         <v/>
       </c>
     </row>

</xml_diff>